<commit_message>
procesar dossier (sin probar)
</commit_message>
<xml_diff>
--- a/ROADMAP_CENTAURO_v2.0.xlsx
+++ b/ROADMAP_CENTAURO_v2.0.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gplaneta.sharepoint.com/sites/BIPOWER/Shared Documents/General/PBI/PROYECTOS/Proyecto_Centauro/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="48" documentId="11_504E058A55DF212521F5348C8936E95C98CE57CC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6DDA0F26-C76C-445F-BE42-8601B87960FE}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1. Resumen Ejecutivo" sheetId="1" r:id="rId1"/>
@@ -16,12 +22,12 @@
     <sheet name="7. Análisis de Costes" sheetId="7" r:id="rId7"/>
     <sheet name="8. RAG - Buenas Prácticas" sheetId="8" r:id="rId8"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="312">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="318">
   <si>
     <t>Métrica</t>
   </si>
@@ -290,9 +296,6 @@
     <t>Feedback Personalizado por Asesor</t>
   </si>
   <si>
-    <t>Exportación a Google Sheets</t>
-  </si>
-  <si>
     <t>Integración con CRM</t>
   </si>
   <si>
@@ -317,9 +320,6 @@
     <t>Generar recomendaciones específicas según historial: 'En tus últimas 3 llamadas, tu cierre promedia 2.5/5'</t>
   </si>
   <si>
-    <t>Subir reportes automáticamente a Google Sheets para análisis colaborativo</t>
-  </si>
-  <si>
     <t>Sincronizar con Salesforce/HubSpot: Actualizar oportunidad con nota de llamada</t>
   </si>
   <si>
@@ -344,9 +344,6 @@
     <t>Alto - Personalización feedback</t>
   </si>
   <si>
-    <t>Medio - Facilita colaboración</t>
-  </si>
-  <si>
     <t>Alto - Integración ecosistema</t>
   </si>
   <si>
@@ -371,9 +368,6 @@
     <t>Pandas + agregaciones</t>
   </si>
   <si>
-    <t>gspread (Google Sheets API)</t>
-  </si>
-  <si>
     <t>API REST del CRM</t>
   </si>
   <si>
@@ -957,13 +951,43 @@
   </si>
   <si>
     <t>Anti-patrón: cierre débil sin compromiso</t>
+  </si>
+  <si>
+    <t>Inclusión de Dossiers de Programa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se debe procesar la información de los dossiers de Programa usando el script procesar_dossiers en el directorio del Proyecto </t>
+  </si>
+  <si>
+    <t>Alto- mejora la información del RAG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Python input() </t>
+  </si>
+  <si>
+    <t>Input de contexto del asesor al agente</t>
+  </si>
+  <si>
+    <t>Crear la opción de que el asesor pueda ingresar parte de información/contexto de forma manual al Agente. Se debe crear un agente especializado que reciba ese input</t>
+  </si>
+  <si>
+    <t>Alto- Mejora la contextualización del Chatbot en general</t>
+  </si>
+  <si>
+    <t>Python + API</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reparar el Orquestador </t>
+  </si>
+  <si>
+    <t>Asegurar que el orquestador de agentes funcione, porque realmente lo esta haciendo todo el orquestador (orchestrator.py)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -988,7 +1012,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -1011,13 +1035,43 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -1026,13 +1080,38 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
+<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
+<FeaturePropertyBags xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
+  <bag type="Checkbox"/>
+  <bag type="XFControls">
+    <bagId k="CellControl">0</bagId>
+  </bag>
+  <bag type="XFComplement">
+    <bagId k="XFControls">1</bagId>
+  </bag>
+  <bag type="XFComplements" extRef="XFComplementsMapperExtRef">
+    <a k="MappedFeaturePropertyBags">
+      <bagId>2</bagId>
+    </a>
+  </bag>
+</FeaturePropertyBags>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1070,7 +1149,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -1104,6 +1183,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -1138,9 +1218,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1313,15 +1394,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B10"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30.7109375" customWidth="1"/>
     <col min="2" max="2" width="70.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1329,7 +1410,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -1337,7 +1418,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1345,7 +1426,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -1353,7 +1434,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -1361,7 +1442,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -1369,7 +1450,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -1377,7 +1458,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -1385,7 +1466,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="9" spans="1:2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -1393,7 +1474,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>10</v>
       </c>
@@ -1407,9 +1488,9 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E14"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.7109375" customWidth="1"/>
     <col min="2" max="2" width="15.7109375" customWidth="1"/>
@@ -1418,7 +1499,7 @@
     <col min="5" max="5" width="15.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>20</v>
       </c>
@@ -1435,12 +1516,12 @@
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>25</v>
       </c>
-      <c r="B2" t="s">
-        <v>38</v>
+      <c r="B2" s="2" t="b">
+        <v>1</v>
       </c>
       <c r="C2" t="s">
         <v>39</v>
@@ -1452,12 +1533,12 @@
         <v>65</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>26</v>
       </c>
-      <c r="B3" t="s">
-        <v>38</v>
+      <c r="B3" s="2" t="b">
+        <v>1</v>
       </c>
       <c r="C3" t="s">
         <v>40</v>
@@ -1469,12 +1550,12 @@
         <v>66</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>27</v>
       </c>
-      <c r="B4" t="s">
-        <v>38</v>
+      <c r="B4" s="2" t="b">
+        <v>1</v>
       </c>
       <c r="C4" t="s">
         <v>41</v>
@@ -1486,12 +1567,12 @@
         <v>67</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>28</v>
       </c>
-      <c r="B5" t="s">
-        <v>38</v>
+      <c r="B5" s="2" t="b">
+        <v>1</v>
       </c>
       <c r="C5" t="s">
         <v>42</v>
@@ -1503,12 +1584,12 @@
         <v>68</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>29</v>
       </c>
-      <c r="B6" t="s">
-        <v>38</v>
+      <c r="B6" s="2" t="b">
+        <v>1</v>
       </c>
       <c r="C6" t="s">
         <v>43</v>
@@ -1520,12 +1601,12 @@
         <v>68</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>30</v>
       </c>
-      <c r="B7" t="s">
-        <v>38</v>
+      <c r="B7" s="2" t="b">
+        <v>1</v>
       </c>
       <c r="C7" t="s">
         <v>44</v>
@@ -1537,12 +1618,12 @@
         <v>69</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>31</v>
       </c>
-      <c r="B8" t="s">
-        <v>38</v>
+      <c r="B8" s="2" t="b">
+        <v>1</v>
       </c>
       <c r="C8" t="s">
         <v>45</v>
@@ -1554,12 +1635,12 @@
         <v>67</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>32</v>
       </c>
-      <c r="B9" t="s">
-        <v>38</v>
+      <c r="B9" s="2" t="b">
+        <v>1</v>
       </c>
       <c r="C9" t="s">
         <v>46</v>
@@ -1571,12 +1652,12 @@
         <v>68</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>33</v>
       </c>
-      <c r="B10" t="s">
-        <v>38</v>
+      <c r="B10" s="2" t="b">
+        <v>1</v>
       </c>
       <c r="C10" t="s">
         <v>47</v>
@@ -1588,12 +1669,12 @@
         <v>70</v>
       </c>
     </row>
-    <row r="11" spans="1:5">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>34</v>
       </c>
-      <c r="B11" t="s">
-        <v>38</v>
+      <c r="B11" s="2" t="b">
+        <v>1</v>
       </c>
       <c r="C11" t="s">
         <v>48</v>
@@ -1605,12 +1686,12 @@
         <v>71</v>
       </c>
     </row>
-    <row r="12" spans="1:5">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>35</v>
       </c>
-      <c r="B12" t="s">
-        <v>38</v>
+      <c r="B12" s="2" t="b">
+        <v>1</v>
       </c>
       <c r="C12" t="s">
         <v>49</v>
@@ -1622,12 +1703,12 @@
         <v>66</v>
       </c>
     </row>
-    <row r="13" spans="1:5">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>36</v>
       </c>
-      <c r="B13" t="s">
-        <v>38</v>
+      <c r="B13" s="2" t="b">
+        <v>1</v>
       </c>
       <c r="C13" t="s">
         <v>50</v>
@@ -1639,12 +1720,12 @@
         <v>66</v>
       </c>
     </row>
-    <row r="14" spans="1:5">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>37</v>
       </c>
-      <c r="B14" t="s">
-        <v>38</v>
+      <c r="B14" s="2" t="b">
+        <v>1</v>
       </c>
       <c r="C14" t="s">
         <v>51</v>
@@ -1662,9 +1743,9 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F10"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:G12"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
     <col min="2" max="2" width="35.7109375" customWidth="1"/>
@@ -1674,7 +1755,7 @@
     <col min="6" max="6" width="30.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>73</v>
       </c>
@@ -1693,185 +1774,253 @@
       <c r="F1" s="1" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="2" spans="1:6">
+      <c r="G1" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>79</v>
       </c>
       <c r="B2" t="s">
-        <v>82</v>
-      </c>
-      <c r="C2" t="s">
-        <v>91</v>
-      </c>
-      <c r="D2">
-        <v>5</v>
-      </c>
-      <c r="E2" t="s">
-        <v>100</v>
-      </c>
-      <c r="F2" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
+        <v>316</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>317</v>
+      </c>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="6"/>
+    </row>
+    <row r="3" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>79</v>
       </c>
       <c r="B3" t="s">
-        <v>83</v>
-      </c>
-      <c r="C3" t="s">
-        <v>92</v>
+        <v>82</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>90</v>
       </c>
       <c r="D3">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E3" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="F3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
+        <v>106</v>
+      </c>
+      <c r="G3" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>79</v>
       </c>
       <c r="B4" t="s">
+        <v>83</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="D4">
+        <v>2</v>
+      </c>
+      <c r="E4" t="s">
+        <v>99</v>
+      </c>
+      <c r="F4" t="s">
+        <v>107</v>
+      </c>
+      <c r="G4" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>79</v>
+      </c>
+      <c r="B5" t="s">
         <v>84</v>
       </c>
-      <c r="C4" t="s">
-        <v>93</v>
-      </c>
-      <c r="D4">
+      <c r="C5" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="D5">
         <v>10</v>
       </c>
-      <c r="E4" t="s">
-        <v>102</v>
-      </c>
-      <c r="F4" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6">
-      <c r="A5" t="s">
-        <v>80</v>
-      </c>
-      <c r="B5" t="s">
-        <v>85</v>
-      </c>
-      <c r="C5" t="s">
-        <v>94</v>
-      </c>
-      <c r="D5">
-        <v>3</v>
-      </c>
       <c r="E5" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="F5" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6">
+        <v>108</v>
+      </c>
+      <c r="G5" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>80</v>
       </c>
       <c r="B6" t="s">
-        <v>86</v>
-      </c>
-      <c r="C6" t="s">
-        <v>95</v>
+        <v>308</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>309</v>
       </c>
       <c r="D6">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E6" t="s">
-        <v>104</v>
+        <v>310</v>
       </c>
       <c r="F6" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6">
+        <v>311</v>
+      </c>
+      <c r="G6" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>80</v>
       </c>
       <c r="B7" t="s">
-        <v>87</v>
-      </c>
-      <c r="C7" t="s">
-        <v>96</v>
+        <v>312</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>313</v>
       </c>
       <c r="D7">
         <v>3</v>
       </c>
       <c r="E7" t="s">
-        <v>105</v>
+        <v>314</v>
       </c>
       <c r="F7" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6">
+        <v>315</v>
+      </c>
+      <c r="G7" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>80</v>
       </c>
       <c r="B8" t="s">
+        <v>85</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="D8">
+        <v>3</v>
+      </c>
+      <c r="E8" t="s">
+        <v>101</v>
+      </c>
+      <c r="F8" t="s">
+        <v>109</v>
+      </c>
+      <c r="G8" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>80</v>
+      </c>
+      <c r="B9" t="s">
+        <v>86</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="D9">
+        <v>7</v>
+      </c>
+      <c r="E9" t="s">
+        <v>102</v>
+      </c>
+      <c r="F9" t="s">
+        <v>110</v>
+      </c>
+      <c r="G9" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>80</v>
+      </c>
+      <c r="B10" t="s">
+        <v>87</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="D10">
+        <v>3</v>
+      </c>
+      <c r="E10" t="s">
+        <v>103</v>
+      </c>
+      <c r="F10" t="s">
+        <v>111</v>
+      </c>
+      <c r="G10" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>80</v>
+      </c>
+      <c r="B11" t="s">
         <v>88</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C11" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D11">
+        <v>5</v>
+      </c>
+      <c r="E11" t="s">
+        <v>104</v>
+      </c>
+      <c r="F11" t="s">
+        <v>112</v>
+      </c>
+      <c r="G11" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>81</v>
+      </c>
+      <c r="B12" t="s">
+        <v>89</v>
+      </c>
+      <c r="C12" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="D8">
-        <v>5</v>
-      </c>
-      <c r="E8" t="s">
-        <v>106</v>
-      </c>
-      <c r="F8" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6">
-      <c r="A9" t="s">
-        <v>81</v>
-      </c>
-      <c r="B9" t="s">
-        <v>89</v>
-      </c>
-      <c r="C9" t="s">
-        <v>98</v>
-      </c>
-      <c r="D9">
-        <v>2</v>
-      </c>
-      <c r="E9" t="s">
-        <v>107</v>
-      </c>
-      <c r="F9" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6">
-      <c r="A10" t="s">
-        <v>81</v>
-      </c>
-      <c r="B10" t="s">
-        <v>90</v>
-      </c>
-      <c r="C10" t="s">
-        <v>99</v>
-      </c>
-      <c r="D10">
+      <c r="D12">
         <v>8</v>
       </c>
-      <c r="E10" t="s">
-        <v>108</v>
-      </c>
-      <c r="F10" t="s">
-        <v>117</v>
+      <c r="E12" t="s">
+        <v>105</v>
+      </c>
+      <c r="F12" t="s">
+        <v>113</v>
+      </c>
+      <c r="G12" s="2" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1880,9 +2029,9 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30.7109375" customWidth="1"/>
     <col min="2" max="2" width="70.7109375" customWidth="1"/>
@@ -1891,154 +2040,154 @@
     <col min="5" max="5" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>20</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="B2" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="C2" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="D2" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="E2" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="B3" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="C3" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="D3" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="E3" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="B4" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="C4" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="D4" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="E4" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="B5" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="C5" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="D5" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="E5" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="B6" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="C6" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="D6" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="E6" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="B7" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="C7" t="s">
+        <v>138</v>
+      </c>
+      <c r="D7" t="s">
         <v>142</v>
-      </c>
-      <c r="D7" t="s">
-        <v>146</v>
       </c>
       <c r="E7" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="B8" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C8" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="D8" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="E8" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="B9" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="C9" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="D9" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="E9" t="s">
         <v>80</v>
@@ -2050,9 +2199,9 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="40.7109375" customWidth="1"/>
     <col min="2" max="2" width="80.7109375" customWidth="1"/>
@@ -2061,7 +2210,7 @@
     <col min="5" max="5" width="15.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>23</v>
       </c>
@@ -2072,160 +2221,160 @@
         <v>78</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="B2" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="C2" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="D2" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="E2">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="B3" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="C3" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="D3" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="E3">
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="B4" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="C4" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="D4" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="E4">
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="B5" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="C5" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="D5" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="E5">
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="B6" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="C6" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="D6" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="E6">
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="B7" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="C7" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="D7" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="E7">
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="B8" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="C8" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="D8" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="E8">
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="B9" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="C9" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D9" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="E9">
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="B10" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="C10" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D10" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="E10">
         <v>12</v>
@@ -2237,9 +2386,9 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:F14"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
     <col min="2" max="2" width="35.7109375" customWidth="1"/>
@@ -2247,284 +2396,284 @@
     <col min="6" max="6" width="25.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>21</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>189</v>
+      </c>
+      <c r="B2" t="s">
         <v>193</v>
       </c>
-      <c r="B2" t="s">
-        <v>197</v>
-      </c>
       <c r="C2" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="D2" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="E2" t="s">
         <v>38</v>
       </c>
       <c r="F2" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="B3" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="C3" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="D3" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="E3" t="s">
         <v>38</v>
       </c>
       <c r="F3" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="B4" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="C4" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="D4" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="E4" t="s">
         <v>38</v>
       </c>
       <c r="F4" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="B5" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="C5" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="D5" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="E5" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="F5" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="B6" t="s">
         <v>84</v>
       </c>
       <c r="C6" t="s">
+        <v>207</v>
+      </c>
+      <c r="D6" t="s">
+        <v>207</v>
+      </c>
+      <c r="E6" t="s">
+        <v>215</v>
+      </c>
+      <c r="F6" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>190</v>
+      </c>
+      <c r="B7" t="s">
+        <v>197</v>
+      </c>
+      <c r="C7" t="s">
+        <v>207</v>
+      </c>
+      <c r="D7" t="s">
+        <v>208</v>
+      </c>
+      <c r="E7" t="s">
+        <v>215</v>
+      </c>
+      <c r="F7" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>190</v>
+      </c>
+      <c r="B8" t="s">
+        <v>198</v>
+      </c>
+      <c r="C8" t="s">
+        <v>207</v>
+      </c>
+      <c r="D8" t="s">
+        <v>208</v>
+      </c>
+      <c r="E8" t="s">
+        <v>215</v>
+      </c>
+      <c r="F8" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>191</v>
+      </c>
+      <c r="B9" t="s">
+        <v>199</v>
+      </c>
+      <c r="C9" t="s">
+        <v>208</v>
+      </c>
+      <c r="D9" t="s">
+        <v>209</v>
+      </c>
+      <c r="E9" t="s">
+        <v>215</v>
+      </c>
+      <c r="F9" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>191</v>
+      </c>
+      <c r="B10" t="s">
+        <v>200</v>
+      </c>
+      <c r="C10" t="s">
+        <v>208</v>
+      </c>
+      <c r="D10" t="s">
+        <v>209</v>
+      </c>
+      <c r="E10" t="s">
+        <v>215</v>
+      </c>
+      <c r="F10" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>191</v>
+      </c>
+      <c r="B11" t="s">
+        <v>201</v>
+      </c>
+      <c r="C11" t="s">
+        <v>209</v>
+      </c>
+      <c r="D11" t="s">
+        <v>209</v>
+      </c>
+      <c r="E11" t="s">
+        <v>215</v>
+      </c>
+      <c r="F11" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>192</v>
+      </c>
+      <c r="B12" t="s">
+        <v>202</v>
+      </c>
+      <c r="C12" t="s">
+        <v>210</v>
+      </c>
+      <c r="D12" t="s">
         <v>211</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E12" t="s">
+        <v>215</v>
+      </c>
+      <c r="F12" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>192</v>
+      </c>
+      <c r="B13" t="s">
+        <v>203</v>
+      </c>
+      <c r="C13" t="s">
         <v>211</v>
       </c>
-      <c r="E6" t="s">
-        <v>219</v>
-      </c>
-      <c r="F6" t="s">
+      <c r="D13" t="s">
+        <v>212</v>
+      </c>
+      <c r="E13" t="s">
+        <v>215</v>
+      </c>
+      <c r="F13" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
-      <c r="A7" t="s">
-        <v>194</v>
-      </c>
-      <c r="B7" t="s">
-        <v>201</v>
-      </c>
-      <c r="C7" t="s">
-        <v>211</v>
-      </c>
-      <c r="D7" t="s">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>192</v>
+      </c>
+      <c r="B14" t="s">
+        <v>204</v>
+      </c>
+      <c r="C14" t="s">
         <v>212</v>
       </c>
-      <c r="E7" t="s">
-        <v>219</v>
-      </c>
-      <c r="F7" t="s">
+      <c r="D14" t="s">
+        <v>213</v>
+      </c>
+      <c r="E14" t="s">
+        <v>215</v>
+      </c>
+      <c r="F14" t="s">
         <v>223</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6">
-      <c r="A8" t="s">
-        <v>194</v>
-      </c>
-      <c r="B8" t="s">
-        <v>202</v>
-      </c>
-      <c r="C8" t="s">
-        <v>211</v>
-      </c>
-      <c r="D8" t="s">
-        <v>212</v>
-      </c>
-      <c r="E8" t="s">
-        <v>219</v>
-      </c>
-      <c r="F8" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6">
-      <c r="A9" t="s">
-        <v>195</v>
-      </c>
-      <c r="B9" t="s">
-        <v>203</v>
-      </c>
-      <c r="C9" t="s">
-        <v>212</v>
-      </c>
-      <c r="D9" t="s">
-        <v>213</v>
-      </c>
-      <c r="E9" t="s">
-        <v>219</v>
-      </c>
-      <c r="F9" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6">
-      <c r="A10" t="s">
-        <v>195</v>
-      </c>
-      <c r="B10" t="s">
-        <v>204</v>
-      </c>
-      <c r="C10" t="s">
-        <v>212</v>
-      </c>
-      <c r="D10" t="s">
-        <v>213</v>
-      </c>
-      <c r="E10" t="s">
-        <v>219</v>
-      </c>
-      <c r="F10" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6">
-      <c r="A11" t="s">
-        <v>195</v>
-      </c>
-      <c r="B11" t="s">
-        <v>205</v>
-      </c>
-      <c r="C11" t="s">
-        <v>213</v>
-      </c>
-      <c r="D11" t="s">
-        <v>213</v>
-      </c>
-      <c r="E11" t="s">
-        <v>219</v>
-      </c>
-      <c r="F11" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6">
-      <c r="A12" t="s">
-        <v>196</v>
-      </c>
-      <c r="B12" t="s">
-        <v>206</v>
-      </c>
-      <c r="C12" t="s">
-        <v>214</v>
-      </c>
-      <c r="D12" t="s">
-        <v>215</v>
-      </c>
-      <c r="E12" t="s">
-        <v>219</v>
-      </c>
-      <c r="F12" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6">
-      <c r="A13" t="s">
-        <v>196</v>
-      </c>
-      <c r="B13" t="s">
-        <v>207</v>
-      </c>
-      <c r="C13" t="s">
-        <v>215</v>
-      </c>
-      <c r="D13" t="s">
-        <v>216</v>
-      </c>
-      <c r="E13" t="s">
-        <v>219</v>
-      </c>
-      <c r="F13" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6">
-      <c r="A14" t="s">
-        <v>196</v>
-      </c>
-      <c r="B14" t="s">
-        <v>208</v>
-      </c>
-      <c r="C14" t="s">
-        <v>216</v>
-      </c>
-      <c r="D14" t="s">
-        <v>217</v>
-      </c>
-      <c r="E14" t="s">
-        <v>219</v>
-      </c>
-      <c r="F14" t="s">
-        <v>227</v>
       </c>
     </row>
   </sheetData>
@@ -2533,172 +2682,172 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="45.7109375" customWidth="1"/>
     <col min="2" max="2" width="20.7109375" customWidth="1"/>
     <col min="3" max="3" width="70.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>227</v>
+      </c>
+      <c r="B2" t="s">
+        <v>241</v>
+      </c>
+      <c r="C2" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>228</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>229</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" t="s">
-        <v>231</v>
-      </c>
-      <c r="B2" t="s">
-        <v>245</v>
-      </c>
-      <c r="C2" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" t="s">
-        <v>232</v>
       </c>
       <c r="B3" t="s">
         <v>66</v>
       </c>
       <c r="C3" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="B4" t="s">
         <v>66</v>
       </c>
       <c r="C4" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>230</v>
+      </c>
+      <c r="B5" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>231</v>
+      </c>
+      <c r="B7" t="s">
+        <v>242</v>
+      </c>
+      <c r="C7" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>232</v>
+      </c>
+      <c r="B8" t="s">
+        <v>243</v>
+      </c>
+      <c r="C8" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>233</v>
+      </c>
+      <c r="B9" t="s">
+        <v>244</v>
+      </c>
+      <c r="C9" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>234</v>
-      </c>
-      <c r="B5" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3">
-      <c r="A7" t="s">
-        <v>235</v>
-      </c>
-      <c r="B7" t="s">
-        <v>246</v>
-      </c>
-      <c r="C7" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3">
-      <c r="A8" t="s">
-        <v>236</v>
-      </c>
-      <c r="B8" t="s">
-        <v>247</v>
-      </c>
-      <c r="C8" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3">
-      <c r="A9" t="s">
-        <v>237</v>
-      </c>
-      <c r="B9" t="s">
-        <v>248</v>
-      </c>
-      <c r="C9" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3">
-      <c r="A10" t="s">
-        <v>238</v>
       </c>
       <c r="B10" t="s">
         <v>66</v>
       </c>
       <c r="C10" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="B11" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="C11" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
       <c r="B12" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="C12" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="B13" t="s">
         <v>66</v>
       </c>
       <c r="C13" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="B14" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
       <c r="B16" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="C16" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B17" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="C17" t="s">
-        <v>265</v>
+        <v>261</v>
       </c>
     </row>
   </sheetData>
@@ -2707,9 +2856,9 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:E12"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.7109375" customWidth="1"/>
     <col min="2" max="2" width="20.7109375" customWidth="1"/>
@@ -2718,208 +2867,208 @@
     <col min="5" max="5" width="50.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>266</v>
       </c>
-      <c r="B1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>267</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="B2" t="s">
+        <v>272</v>
+      </c>
+      <c r="C2" t="s">
+        <v>275</v>
+      </c>
+      <c r="D2" t="s">
+        <v>286</v>
+      </c>
+      <c r="E2" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>267</v>
+      </c>
+      <c r="B3" t="s">
+        <v>273</v>
+      </c>
+      <c r="C3" t="s">
+        <v>276</v>
+      </c>
+      <c r="D3" t="s">
+        <v>287</v>
+      </c>
+      <c r="E3" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>267</v>
+      </c>
+      <c r="B4" t="s">
+        <v>274</v>
+      </c>
+      <c r="C4" t="s">
+        <v>277</v>
+      </c>
+      <c r="D4" t="s">
+        <v>288</v>
+      </c>
+      <c r="E4" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>268</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="B5" t="s">
+        <v>272</v>
+      </c>
+      <c r="C5" t="s">
+        <v>278</v>
+      </c>
+      <c r="D5" t="s">
+        <v>289</v>
+      </c>
+      <c r="E5" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>268</v>
+      </c>
+      <c r="B6" t="s">
+        <v>274</v>
+      </c>
+      <c r="C6" t="s">
+        <v>279</v>
+      </c>
+      <c r="D6" t="s">
+        <v>290</v>
+      </c>
+      <c r="E6" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>269</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="B7" t="s">
+        <v>272</v>
+      </c>
+      <c r="C7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D7" t="s">
+        <v>291</v>
+      </c>
+      <c r="E7" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>269</v>
+      </c>
+      <c r="B8" t="s">
+        <v>274</v>
+      </c>
+      <c r="C8" t="s">
+        <v>281</v>
+      </c>
+      <c r="D8" t="s">
+        <v>292</v>
+      </c>
+      <c r="E8" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>270</v>
       </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2" t="s">
+      <c r="B9" t="s">
+        <v>272</v>
+      </c>
+      <c r="C9" t="s">
+        <v>282</v>
+      </c>
+      <c r="D9" t="s">
+        <v>293</v>
+      </c>
+      <c r="E9" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>270</v>
+      </c>
+      <c r="B10" t="s">
+        <v>274</v>
+      </c>
+      <c r="C10" t="s">
+        <v>283</v>
+      </c>
+      <c r="D10" t="s">
+        <v>294</v>
+      </c>
+      <c r="E10" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>271</v>
       </c>
-      <c r="B2" t="s">
-        <v>276</v>
-      </c>
-      <c r="C2" t="s">
-        <v>279</v>
-      </c>
-      <c r="D2" t="s">
-        <v>290</v>
-      </c>
-      <c r="E2" t="s">
-        <v>301</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5">
-      <c r="A3" t="s">
+      <c r="B11" t="s">
+        <v>272</v>
+      </c>
+      <c r="C11" t="s">
+        <v>284</v>
+      </c>
+      <c r="D11" t="s">
+        <v>295</v>
+      </c>
+      <c r="E11" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>271</v>
       </c>
-      <c r="B3" t="s">
-        <v>277</v>
-      </c>
-      <c r="C3" t="s">
-        <v>280</v>
-      </c>
-      <c r="D3" t="s">
-        <v>291</v>
-      </c>
-      <c r="E3" t="s">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5">
-      <c r="A4" t="s">
-        <v>271</v>
-      </c>
-      <c r="B4" t="s">
-        <v>278</v>
-      </c>
-      <c r="C4" t="s">
-        <v>281</v>
-      </c>
-      <c r="D4" t="s">
-        <v>292</v>
-      </c>
-      <c r="E4" t="s">
-        <v>303</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5">
-      <c r="A5" t="s">
-        <v>272</v>
-      </c>
-      <c r="B5" t="s">
-        <v>276</v>
-      </c>
-      <c r="C5" t="s">
-        <v>282</v>
-      </c>
-      <c r="D5" t="s">
-        <v>293</v>
-      </c>
-      <c r="E5" t="s">
-        <v>304</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5">
-      <c r="A6" t="s">
-        <v>272</v>
-      </c>
-      <c r="B6" t="s">
-        <v>278</v>
-      </c>
-      <c r="C6" t="s">
-        <v>283</v>
-      </c>
-      <c r="D6" t="s">
-        <v>294</v>
-      </c>
-      <c r="E6" t="s">
-        <v>305</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5">
-      <c r="A7" t="s">
-        <v>273</v>
-      </c>
-      <c r="B7" t="s">
-        <v>276</v>
-      </c>
-      <c r="C7" t="s">
-        <v>284</v>
-      </c>
-      <c r="D7" t="s">
-        <v>295</v>
-      </c>
-      <c r="E7" t="s">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5">
-      <c r="A8" t="s">
-        <v>273</v>
-      </c>
-      <c r="B8" t="s">
-        <v>278</v>
-      </c>
-      <c r="C8" t="s">
+      <c r="B12" t="s">
+        <v>274</v>
+      </c>
+      <c r="C12" t="s">
         <v>285</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D12" t="s">
         <v>296</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E12" t="s">
         <v>307</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5">
-      <c r="A9" t="s">
-        <v>274</v>
-      </c>
-      <c r="B9" t="s">
-        <v>276</v>
-      </c>
-      <c r="C9" t="s">
-        <v>286</v>
-      </c>
-      <c r="D9" t="s">
-        <v>297</v>
-      </c>
-      <c r="E9" t="s">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5">
-      <c r="A10" t="s">
-        <v>274</v>
-      </c>
-      <c r="B10" t="s">
-        <v>278</v>
-      </c>
-      <c r="C10" t="s">
-        <v>287</v>
-      </c>
-      <c r="D10" t="s">
-        <v>298</v>
-      </c>
-      <c r="E10" t="s">
-        <v>309</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5">
-      <c r="A11" t="s">
-        <v>275</v>
-      </c>
-      <c r="B11" t="s">
-        <v>276</v>
-      </c>
-      <c r="C11" t="s">
-        <v>288</v>
-      </c>
-      <c r="D11" t="s">
-        <v>299</v>
-      </c>
-      <c r="E11" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5">
-      <c r="A12" t="s">
-        <v>275</v>
-      </c>
-      <c r="B12" t="s">
-        <v>278</v>
-      </c>
-      <c r="C12" t="s">
-        <v>289</v>
-      </c>
-      <c r="D12" t="s">
-        <v>300</v>
-      </c>
-      <c r="E12" t="s">
-        <v>311</v>
       </c>
     </row>
   </sheetData>
@@ -2928,6 +3077,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="396b9688-3d64-4f4f-b40d-59fd809f50b1" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e4f8e1ef-7590-4615-a0b0-41d92864fb7e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A62BD1A1B5CAC249A95BCCCA1576DD25" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="95d80e3e9b41a0cd0f31651385762a39">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="e4f8e1ef-7590-4615-a0b0-41d92864fb7e" xmlns:ns3="396b9688-3d64-4f4f-b40d-59fd809f50b1" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0c785e827d86c3245c0f7c251e0c72c1" ns2:_="" ns3:_="">
     <xsd:import namespace="e4f8e1ef-7590-4615-a0b0-41d92864fb7e"/>
@@ -3162,34 +3331,40 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="396b9688-3d64-4f4f-b40d-59fd809f50b1" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e4f8e1ef-7590-4615-a0b0-41d92864fb7e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{01F79570-1C8D-46A0-B328-3C974A919A6F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BF3EE484-6495-4CA4-BA24-055A9C2DA68A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="396b9688-3d64-4f4f-b40d-59fd809f50b1"/>
+    <ds:schemaRef ds:uri="e4f8e1ef-7590-4615-a0b0-41d92864fb7e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{715A098D-F1BB-49A5-A110-A0EC96ECC1ED}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{715A098D-F1BB-49A5-A110-A0EC96ECC1ED}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BF3EE484-6495-4CA4-BA24-055A9C2DA68A}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{01F79570-1C8D-46A0-B328-3C974A919A6F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="e4f8e1ef-7590-4615-a0b0-41d92864fb7e"/>
+    <ds:schemaRef ds:uri="396b9688-3d64-4f4f-b40d-59fd809f50b1"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>